<commit_message>
actualizacion de nuevo registro, letras con mala redaccion funcionando
</commit_message>
<xml_diff>
--- a/Informe.xlsx
+++ b/Informe.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1091"/>
+  <dimension ref="A1:I1095"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15952,8 +15952,16 @@
           <t>3722</t>
         </is>
       </c>
-      <c r="B398" t="inlineStr"/>
-      <c r="C398" t="inlineStr"/>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>ccastro@semana.com mjimenez@cmmlegal.co</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>cundinamarca</t>
+        </is>
+      </c>
       <c r="D398" t="inlineStr">
         <is>
           <t>26102023447394</t>
@@ -15971,7 +15979,7 @@
       </c>
       <c r="G398" t="inlineStr">
         <is>
-          <t>Enviado</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H398" t="inlineStr">
@@ -23508,7 +23516,11 @@
           <t>114</t>
         </is>
       </c>
-      <c r="B586" t="inlineStr"/>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>ingrith1183@hotmail.com duran.carrillo@hotmail.com</t>
+        </is>
+      </c>
       <c r="C586" t="inlineStr"/>
       <c r="D586" t="inlineStr">
         <is>
@@ -23522,7 +23534,7 @@
       </c>
       <c r="F586" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G586" t="inlineStr">
@@ -26091,7 +26103,7 @@
       </c>
       <c r="F649" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G649" t="inlineStr">
@@ -28068,7 +28080,7 @@
       </c>
       <c r="G697" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="H697" t="inlineStr">
@@ -30330,7 +30342,7 @@
       </c>
       <c r="G751" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="H751" t="inlineStr">
@@ -44407,7 +44419,7 @@
       </c>
       <c r="F1061" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G1061" t="inlineStr">
@@ -44966,7 +44978,7 @@
       </c>
       <c r="F1074" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G1074" t="inlineStr">
@@ -45218,8 +45230,16 @@
           <t>Enviado</t>
         </is>
       </c>
-      <c r="F1080" t="inlineStr"/>
-      <c r="G1080" t="inlineStr"/>
+      <c r="F1080" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1080" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1080" t="inlineStr"/>
       <c r="I1080" t="inlineStr">
         <is>
@@ -45253,8 +45273,16 @@
           <t>Enviado</t>
         </is>
       </c>
-      <c r="F1081" t="inlineStr"/>
-      <c r="G1081" t="inlineStr"/>
+      <c r="F1081" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1081" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1081" t="inlineStr"/>
       <c r="I1081" t="inlineStr">
         <is>
@@ -45288,8 +45316,16 @@
           <t>Enviado</t>
         </is>
       </c>
-      <c r="F1082" t="inlineStr"/>
-      <c r="G1082" t="inlineStr"/>
+      <c r="F1082" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1082" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1082" t="inlineStr"/>
       <c r="I1082" t="inlineStr">
         <is>
@@ -45323,8 +45359,16 @@
           <t>Enviado</t>
         </is>
       </c>
-      <c r="F1083" t="inlineStr"/>
-      <c r="G1083" t="inlineStr"/>
+      <c r="F1083" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1083" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1083" t="inlineStr"/>
       <c r="I1083" t="inlineStr">
         <is>
@@ -45358,8 +45402,16 @@
           <t>Enviado</t>
         </is>
       </c>
-      <c r="F1084" t="inlineStr"/>
-      <c r="G1084" t="inlineStr"/>
+      <c r="F1084" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1084" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1084" t="inlineStr"/>
       <c r="I1084" t="inlineStr">
         <is>
@@ -45389,8 +45441,16 @@
           <t>Enviado</t>
         </is>
       </c>
-      <c r="F1085" t="inlineStr"/>
-      <c r="G1085" t="inlineStr"/>
+      <c r="F1085" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1085" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1085" t="inlineStr"/>
       <c r="I1085" t="inlineStr">
         <is>
@@ -45424,8 +45484,16 @@
           <t>Enviado</t>
         </is>
       </c>
-      <c r="F1086" t="inlineStr"/>
-      <c r="G1086" t="inlineStr"/>
+      <c r="F1086" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1086" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1086" t="inlineStr"/>
       <c r="I1086" t="inlineStr">
         <is>
@@ -45459,8 +45527,16 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F1087" t="inlineStr"/>
-      <c r="G1087" t="inlineStr"/>
+      <c r="F1087" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1087" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1087" t="inlineStr"/>
       <c r="I1087" t="inlineStr">
         <is>
@@ -45494,8 +45570,16 @@
           <t>Enviado</t>
         </is>
       </c>
-      <c r="F1088" t="inlineStr"/>
-      <c r="G1088" t="inlineStr"/>
+      <c r="F1088" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1088" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1088" t="inlineStr"/>
       <c r="I1088" t="inlineStr">
         <is>
@@ -45529,8 +45613,16 @@
           <t>Enviado</t>
         </is>
       </c>
-      <c r="F1089" t="inlineStr"/>
-      <c r="G1089" t="inlineStr"/>
+      <c r="F1089" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1089" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1089" t="inlineStr"/>
       <c r="I1089" t="inlineStr">
         <is>
@@ -45561,11 +45653,19 @@
       </c>
       <c r="E1090" t="inlineStr">
         <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1090" t="inlineStr">
+        <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F1090" t="inlineStr"/>
-      <c r="G1090" t="inlineStr"/>
+      <c r="G1090" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1090" t="inlineStr"/>
       <c r="I1090" t="inlineStr">
         <is>
@@ -45599,12 +45699,192 @@
           <t>Enviado</t>
         </is>
       </c>
-      <c r="F1091" t="inlineStr"/>
-      <c r="G1091" t="inlineStr"/>
+      <c r="F1091" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1091" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1091" t="inlineStr"/>
       <c r="I1091" t="inlineStr">
         <is>
           <t>905</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="inlineStr">
+        <is>
+          <t>530</t>
+        </is>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>albert.tg91@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1092" t="inlineStr">
+        <is>
+          <t>26102023782488</t>
+        </is>
+      </c>
+      <c r="E1092" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1092" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1092" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1092" t="inlineStr"/>
+      <c r="I1092" t="inlineStr">
+        <is>
+          <t>530</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" t="inlineStr">
+        <is>
+          <t>729</t>
+        </is>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>anisam25@hotmail.com santiiagolopezmorales@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1093" t="inlineStr">
+        <is>
+          <t>26102023782701</t>
+        </is>
+      </c>
+      <c r="E1093" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1093" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1093" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1093" t="inlineStr"/>
+      <c r="I1093" t="inlineStr">
+        <is>
+          <t>729</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" t="inlineStr">
+        <is>
+          <t>921</t>
+        </is>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>arturoruizg77@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1094" t="inlineStr">
+        <is>
+          <t>26102023782730</t>
+        </is>
+      </c>
+      <c r="E1094" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1094" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1094" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1094" t="inlineStr"/>
+      <c r="I1094" t="inlineStr">
+        <is>
+          <t>921</t>
+        </is>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" t="inlineStr">
+        <is>
+          <t>884</t>
+        </is>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>yennymarilundiazmez@gmail.com yurybenitezlegal@gmail.com jdjoraquira@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1095" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1095" t="inlineStr">
+        <is>
+          <t>26102023782752</t>
+        </is>
+      </c>
+      <c r="E1095" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1095" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1095" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1095" t="inlineStr"/>
+      <c r="I1095" t="inlineStr">
+        <is>
+          <t>884</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Modificacion visual en css actualizacion en certificados
</commit_message>
<xml_diff>
--- a/Informe.xlsx
+++ b/Informe.xlsx
@@ -13,7 +13,7 @@
     <definedName name="_56F9DC9755BA473782653E2940F9ResponseSheet">"Form1"</definedName>
     <definedName name="_56F9DC9755BA473782653E2940F9SourceDocId">"{5ead13d5-5352-4817-a0e2-9f7def58e808}"</definedName>
   </definedNames>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1" iterate="1"/>
 </workbook>
 </file>
 
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1091"/>
+  <dimension ref="A1:I1168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12959,12 +12959,12 @@
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>Ingresado</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G321" t="inlineStr">
         <is>
-          <t>Enviado</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H321" t="inlineStr">
@@ -17031,7 +17031,7 @@
       </c>
       <c r="F425" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G425" t="inlineStr">
@@ -17277,7 +17277,7 @@
       </c>
       <c r="F431" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G431" t="inlineStr">
@@ -17945,7 +17945,7 @@
       </c>
       <c r="F447" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G447" t="inlineStr">
@@ -17988,7 +17988,7 @@
       </c>
       <c r="F448" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G448" t="inlineStr">
@@ -18230,7 +18230,7 @@
       </c>
       <c r="F454" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G454" t="inlineStr">
@@ -18308,7 +18308,7 @@
       </c>
       <c r="F456" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G456" t="inlineStr">
@@ -18819,7 +18819,7 @@
       </c>
       <c r="F469" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G469" t="inlineStr">
@@ -18863,7 +18863,7 @@
       </c>
       <c r="G470" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="H470" t="inlineStr">
@@ -18897,7 +18897,7 @@
       </c>
       <c r="F471" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G471" t="inlineStr">
@@ -19057,7 +19057,7 @@
       </c>
       <c r="F475" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G475" t="inlineStr">
@@ -19178,7 +19178,7 @@
       </c>
       <c r="F478" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G478" t="inlineStr">
@@ -19689,7 +19689,7 @@
       </c>
       <c r="F491" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G491" t="inlineStr">
@@ -19884,7 +19884,7 @@
       </c>
       <c r="F496" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G496" t="inlineStr">
@@ -20220,7 +20220,7 @@
       </c>
       <c r="F504" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G504" t="inlineStr">
@@ -20337,7 +20337,7 @@
       </c>
       <c r="F507" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G507" t="inlineStr">
@@ -20548,7 +20548,7 @@
       </c>
       <c r="F512" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G512" t="inlineStr">
@@ -20634,7 +20634,7 @@
       </c>
       <c r="F514" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G514" t="inlineStr">
@@ -20677,7 +20677,7 @@
       </c>
       <c r="F515" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G515" t="inlineStr">
@@ -20880,7 +20880,7 @@
       </c>
       <c r="F520" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G520" t="inlineStr">
@@ -22164,7 +22164,7 @@
       </c>
       <c r="F552" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G552" t="inlineStr">
@@ -22207,7 +22207,7 @@
       </c>
       <c r="F553" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G553" t="inlineStr">
@@ -22652,7 +22652,7 @@
       </c>
       <c r="F564" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G564" t="inlineStr">
@@ -22964,7 +22964,7 @@
       </c>
       <c r="F572" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G572" t="inlineStr">
@@ -23928,7 +23928,7 @@
       </c>
       <c r="F596" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G596" t="inlineStr">
@@ -24101,7 +24101,7 @@
       </c>
       <c r="G600" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="H600" t="inlineStr">
@@ -24135,7 +24135,7 @@
       </c>
       <c r="F601" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G601" t="inlineStr">
@@ -24330,7 +24330,7 @@
       </c>
       <c r="F606" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G606" t="inlineStr">
@@ -24369,7 +24369,7 @@
       </c>
       <c r="F607" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G607" t="inlineStr">
@@ -24658,7 +24658,7 @@
       </c>
       <c r="F614" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G614" t="inlineStr">
@@ -24697,7 +24697,7 @@
       </c>
       <c r="F615" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G615" t="inlineStr">
@@ -25064,7 +25064,7 @@
       </c>
       <c r="F624" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G624" t="inlineStr">
@@ -25189,7 +25189,7 @@
       </c>
       <c r="F627" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G627" t="inlineStr">
@@ -25603,7 +25603,7 @@
       </c>
       <c r="F637" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G637" t="inlineStr">
@@ -25970,7 +25970,7 @@
       </c>
       <c r="F646" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G646" t="inlineStr">
@@ -30330,7 +30330,7 @@
       </c>
       <c r="G751" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="H751" t="inlineStr">
@@ -33544,7 +33544,7 @@
       </c>
       <c r="F820" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Ingresado</t>
         </is>
       </c>
       <c r="G820" t="inlineStr">
@@ -36040,7 +36040,7 @@
       </c>
       <c r="G873" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="H873" t="inlineStr">
@@ -36181,7 +36181,7 @@
       </c>
       <c r="G876" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="H876" t="inlineStr">
@@ -36745,7 +36745,7 @@
       </c>
       <c r="G888" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="H888" t="inlineStr">
@@ -36980,7 +36980,7 @@
       </c>
       <c r="G893" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="H893" t="inlineStr">
@@ -37732,7 +37732,7 @@
       </c>
       <c r="G909" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="H909" t="inlineStr">
@@ -39232,7 +39232,7 @@
       </c>
       <c r="G941" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="H941" t="inlineStr">
@@ -39467,7 +39467,7 @@
       </c>
       <c r="G946" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="H946" t="inlineStr">
@@ -40726,7 +40726,7 @@
       </c>
       <c r="G975" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="H975" t="inlineStr"/>
@@ -41156,7 +41156,7 @@
       </c>
       <c r="G985" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="H985" t="inlineStr"/>
@@ -42266,7 +42266,7 @@
       </c>
       <c r="G1011" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="H1011" t="inlineStr"/>
@@ -45218,8 +45218,16 @@
           <t>Enviado</t>
         </is>
       </c>
-      <c r="F1080" t="inlineStr"/>
-      <c r="G1080" t="inlineStr"/>
+      <c r="F1080" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1080" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1080" t="inlineStr"/>
       <c r="I1080" t="inlineStr">
         <is>
@@ -45253,8 +45261,16 @@
           <t>Enviado</t>
         </is>
       </c>
-      <c r="F1081" t="inlineStr"/>
-      <c r="G1081" t="inlineStr"/>
+      <c r="F1081" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1081" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1081" t="inlineStr"/>
       <c r="I1081" t="inlineStr">
         <is>
@@ -45288,8 +45304,16 @@
           <t>Enviado</t>
         </is>
       </c>
-      <c r="F1082" t="inlineStr"/>
-      <c r="G1082" t="inlineStr"/>
+      <c r="F1082" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1082" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1082" t="inlineStr"/>
       <c r="I1082" t="inlineStr">
         <is>
@@ -45323,8 +45347,16 @@
           <t>Enviado</t>
         </is>
       </c>
-      <c r="F1083" t="inlineStr"/>
-      <c r="G1083" t="inlineStr"/>
+      <c r="F1083" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1083" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1083" t="inlineStr"/>
       <c r="I1083" t="inlineStr">
         <is>
@@ -45358,8 +45390,16 @@
           <t>Enviado</t>
         </is>
       </c>
-      <c r="F1084" t="inlineStr"/>
-      <c r="G1084" t="inlineStr"/>
+      <c r="F1084" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1084" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1084" t="inlineStr"/>
       <c r="I1084" t="inlineStr">
         <is>
@@ -45389,8 +45429,16 @@
           <t>Enviado</t>
         </is>
       </c>
-      <c r="F1085" t="inlineStr"/>
-      <c r="G1085" t="inlineStr"/>
+      <c r="F1085" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1085" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1085" t="inlineStr"/>
       <c r="I1085" t="inlineStr">
         <is>
@@ -45424,8 +45472,16 @@
           <t>Enviado</t>
         </is>
       </c>
-      <c r="F1086" t="inlineStr"/>
-      <c r="G1086" t="inlineStr"/>
+      <c r="F1086" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1086" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1086" t="inlineStr"/>
       <c r="I1086" t="inlineStr">
         <is>
@@ -45456,11 +45512,19 @@
       </c>
       <c r="E1087" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F1087" t="inlineStr"/>
-      <c r="G1087" t="inlineStr"/>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1087" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1087" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1087" t="inlineStr"/>
       <c r="I1087" t="inlineStr">
         <is>
@@ -45494,8 +45558,16 @@
           <t>Enviado</t>
         </is>
       </c>
-      <c r="F1088" t="inlineStr"/>
-      <c r="G1088" t="inlineStr"/>
+      <c r="F1088" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1088" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1088" t="inlineStr"/>
       <c r="I1088" t="inlineStr">
         <is>
@@ -45529,8 +45601,16 @@
           <t>Enviado</t>
         </is>
       </c>
-      <c r="F1089" t="inlineStr"/>
-      <c r="G1089" t="inlineStr"/>
+      <c r="F1089" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1089" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1089" t="inlineStr"/>
       <c r="I1089" t="inlineStr">
         <is>
@@ -45561,11 +45641,19 @@
       </c>
       <c r="E1090" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F1090" t="inlineStr"/>
-      <c r="G1090" t="inlineStr"/>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1090" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1090" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1090" t="inlineStr"/>
       <c r="I1090" t="inlineStr">
         <is>
@@ -45599,12 +45687,3323 @@
           <t>Enviado</t>
         </is>
       </c>
-      <c r="F1091" t="inlineStr"/>
-      <c r="G1091" t="inlineStr"/>
+      <c r="F1091" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1091" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="H1091" t="inlineStr"/>
       <c r="I1091" t="inlineStr">
         <is>
           <t>905</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="inlineStr">
+        <is>
+          <t>729</t>
+        </is>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>anisam25@hotmail.com santiiagolopezmorales@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1092" t="inlineStr">
+        <is>
+          <t>26102023782701</t>
+        </is>
+      </c>
+      <c r="E1092" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1092" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1092" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1092" t="inlineStr"/>
+      <c r="I1092" t="inlineStr">
+        <is>
+          <t>729</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" t="inlineStr">
+        <is>
+          <t>921</t>
+        </is>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>arturoruizg77@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1093" t="inlineStr">
+        <is>
+          <t>26102023782730</t>
+        </is>
+      </c>
+      <c r="E1093" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1093" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1093" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1093" t="inlineStr"/>
+      <c r="I1093" t="inlineStr">
+        <is>
+          <t>921</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" t="inlineStr">
+        <is>
+          <t>884</t>
+        </is>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>yennymarilundiazmez@gmail.com yurybenitezlegal@gmail.com jdjoraquira@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1094" t="inlineStr">
+        <is>
+          <t>26102023782752</t>
+        </is>
+      </c>
+      <c r="E1094" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1094" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1094" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1094" t="inlineStr"/>
+      <c r="I1094" t="inlineStr">
+        <is>
+          <t>884</t>
+        </is>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" t="inlineStr">
+        <is>
+          <t>891</t>
+        </is>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>miguel--0108@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1095" t="inlineStr">
+        <is>
+          <t>Santander</t>
+        </is>
+      </c>
+      <c r="D1095" t="inlineStr">
+        <is>
+          <t>26102023785028</t>
+        </is>
+      </c>
+      <c r="E1095" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F1095" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1095" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1095" t="inlineStr"/>
+      <c r="I1095" t="inlineStr">
+        <is>
+          <t>891</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>danilu1703@hotmail.com umv@marval.com.co</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1096" t="inlineStr">
+        <is>
+          <t>26102023787503</t>
+        </is>
+      </c>
+      <c r="E1096" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1096" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1096" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1096" t="inlineStr"/>
+      <c r="I1096" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" t="inlineStr">
+        <is>
+          <t>640</t>
+        </is>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>rinnelly@hotmail.com umv@marval.com.co rin-nelly@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1097" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1097" t="inlineStr">
+        <is>
+          <t>26102023787587</t>
+        </is>
+      </c>
+      <c r="E1097" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1097" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1097" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1097" t="inlineStr"/>
+      <c r="I1097" t="inlineStr">
+        <is>
+          <t>640</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" t="inlineStr">
+        <is>
+          <t>642</t>
+        </is>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>angelalilianavilauribe2@gmail.com umv@marval.com.co</t>
+        </is>
+      </c>
+      <c r="C1098" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1098" t="inlineStr">
+        <is>
+          <t>26102023787610</t>
+        </is>
+      </c>
+      <c r="E1098" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1098" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1098" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1098" t="inlineStr"/>
+      <c r="I1098" t="inlineStr">
+        <is>
+          <t>642</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" t="inlineStr">
+        <is>
+          <t>646</t>
+        </is>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>umv@marval.com.co evamariavar@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1099" t="inlineStr">
+        <is>
+          <t>26102023787631</t>
+        </is>
+      </c>
+      <c r="E1099" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1099" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1099" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1099" t="inlineStr"/>
+      <c r="I1099" t="inlineStr">
+        <is>
+          <t>646</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" t="inlineStr">
+        <is>
+          <t>652</t>
+        </is>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>umv@marval.com.co tomasglpr@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1100" t="inlineStr">
+        <is>
+          <t>26102023787647</t>
+        </is>
+      </c>
+      <c r="E1100" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1100" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1100" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1100" t="inlineStr"/>
+      <c r="I1100" t="inlineStr">
+        <is>
+          <t>652</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" t="inlineStr">
+        <is>
+          <t>656</t>
+        </is>
+      </c>
+      <c r="B1101" t="inlineStr">
+        <is>
+          <t>edilsontrujillo04@gmail.com  umv@marval.com.co</t>
+        </is>
+      </c>
+      <c r="C1101" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1101" t="inlineStr">
+        <is>
+          <t>26102023787661</t>
+        </is>
+      </c>
+      <c r="E1101" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1101" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1101" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1101" t="inlineStr"/>
+      <c r="I1101" t="inlineStr">
+        <is>
+          <t>656</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="B1102" t="inlineStr">
+        <is>
+          <t>camilo95.155@gmail.com operacionesinmobiliarias@proyectosyurbanizaciones.com</t>
+        </is>
+      </c>
+      <c r="C1102" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1102" t="inlineStr">
+        <is>
+          <t>26102023788259</t>
+        </is>
+      </c>
+      <c r="E1102" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1102" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1102" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1102" t="inlineStr"/>
+      <c r="I1102" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" t="inlineStr">
+        <is>
+          <t>749</t>
+        </is>
+      </c>
+      <c r="B1103" t="inlineStr">
+        <is>
+          <t>julii09montoya@gmail.com operacionesinmobiliarias@proyectosyurbanizaciones.com</t>
+        </is>
+      </c>
+      <c r="C1103" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1103" t="inlineStr">
+        <is>
+          <t>26102023788318</t>
+        </is>
+      </c>
+      <c r="E1103" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1103" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1103" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1103" t="inlineStr"/>
+      <c r="I1103" t="inlineStr">
+        <is>
+          <t>749</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" t="inlineStr">
+        <is>
+          <t>763</t>
+        </is>
+      </c>
+      <c r="B1104" t="inlineStr">
+        <is>
+          <t>blancaortiz@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1104" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1104" t="inlineStr">
+        <is>
+          <t>26102023788734</t>
+        </is>
+      </c>
+      <c r="E1104" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F1104" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1104" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1104" t="inlineStr"/>
+      <c r="I1104" t="inlineStr">
+        <is>
+          <t>763</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" t="inlineStr">
+        <is>
+          <t>786</t>
+        </is>
+      </c>
+      <c r="B1105" t="inlineStr">
+        <is>
+          <t>vmojicamanrique@gmail.com wilmar_mm@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1105" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1105" t="inlineStr">
+        <is>
+          <t>26102023789093</t>
+        </is>
+      </c>
+      <c r="E1105" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1105" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1105" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1105" t="inlineStr"/>
+      <c r="I1105" t="inlineStr">
+        <is>
+          <t>786</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" t="inlineStr">
+        <is>
+          <t>834</t>
+        </is>
+      </c>
+      <c r="B1106" t="inlineStr">
+        <is>
+          <t>fernandasl@msn.com</t>
+        </is>
+      </c>
+      <c r="C1106" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1106" t="inlineStr">
+        <is>
+          <t>26102023789179</t>
+        </is>
+      </c>
+      <c r="E1106" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1106" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1106" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1106" t="inlineStr"/>
+      <c r="I1106" t="inlineStr">
+        <is>
+          <t>834</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" t="inlineStr">
+        <is>
+          <t>838</t>
+        </is>
+      </c>
+      <c r="B1107" t="inlineStr">
+        <is>
+          <t>ariverost@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1107" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1107" t="inlineStr">
+        <is>
+          <t>26102023789234</t>
+        </is>
+      </c>
+      <c r="E1107" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1107" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1107" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1107" t="inlineStr"/>
+      <c r="I1107" t="inlineStr">
+        <is>
+          <t>838</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" t="inlineStr">
+        <is>
+          <t>860</t>
+        </is>
+      </c>
+      <c r="B1108" t="inlineStr">
+        <is>
+          <t>lopezcardenasolgalucia@gmail.com rubyvera@gmail.com lopeztere064@gmail.com majlopezv@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1108" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1108" t="inlineStr">
+        <is>
+          <t>26102023789274</t>
+        </is>
+      </c>
+      <c r="E1108" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1108" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1108" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1108" t="inlineStr"/>
+      <c r="I1108" t="inlineStr">
+        <is>
+          <t>860</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" t="inlineStr">
+        <is>
+          <t>943</t>
+        </is>
+      </c>
+      <c r="B1109" t="inlineStr">
+        <is>
+          <t>stpt.elolivarsa@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1109" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1109" t="inlineStr">
+        <is>
+          <t>26102023789592</t>
+        </is>
+      </c>
+      <c r="E1109" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1109" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1109" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1109" t="inlineStr"/>
+      <c r="I1109" t="inlineStr">
+        <is>
+          <t>943</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" t="inlineStr">
+        <is>
+          <t>897</t>
+        </is>
+      </c>
+      <c r="B1110" t="inlineStr">
+        <is>
+          <t>pbogoya@yahoo.com dnlboyaca@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1110" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1110" t="inlineStr">
+        <is>
+          <t>26102023789703</t>
+        </is>
+      </c>
+      <c r="E1110" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1110" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1110" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1110" t="inlineStr"/>
+      <c r="I1110" t="inlineStr">
+        <is>
+          <t>897</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" t="inlineStr">
+        <is>
+          <t>898</t>
+        </is>
+      </c>
+      <c r="B1111" t="inlineStr">
+        <is>
+          <t>acevedoolayamiguel@gmail.com angelesdemaria2104@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1111" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1111" t="inlineStr">
+        <is>
+          <t>26102023789751</t>
+        </is>
+      </c>
+      <c r="E1111" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1111" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1111" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1111" t="inlineStr"/>
+      <c r="I1111" t="inlineStr">
+        <is>
+          <t>898</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" t="inlineStr">
+        <is>
+          <t>917</t>
+        </is>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>williamg0104@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1112" t="inlineStr">
+        <is>
+          <t>26102023789789</t>
+        </is>
+      </c>
+      <c r="E1112" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1112" t="inlineStr">
+        <is>
+          <t>Ingresado</t>
+        </is>
+      </c>
+      <c r="G1112" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1112" t="inlineStr"/>
+      <c r="I1112" t="inlineStr">
+        <is>
+          <t>917</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" t="inlineStr">
+        <is>
+          <t>644</t>
+        </is>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>umv@marval.com.co alejoescribe@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1113" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1113" t="inlineStr">
+        <is>
+          <t>26102023789815</t>
+        </is>
+      </c>
+      <c r="E1113" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1113" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1113" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1113" t="inlineStr"/>
+      <c r="I1113" t="inlineStr">
+        <is>
+          <t>644</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" t="inlineStr">
+        <is>
+          <t>765</t>
+        </is>
+      </c>
+      <c r="B1114" t="inlineStr">
+        <is>
+          <t>dsuarez910@gmail.com operacionesinmobiliarias@proyectosyurbanizaciones.com</t>
+        </is>
+      </c>
+      <c r="C1114" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1114" t="inlineStr">
+        <is>
+          <t>26102023789859</t>
+        </is>
+      </c>
+      <c r="E1114" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1114" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1114" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1114" t="inlineStr"/>
+      <c r="I1114" t="inlineStr">
+        <is>
+          <t>765</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" t="inlineStr">
+        <is>
+          <t>754</t>
+        </is>
+      </c>
+      <c r="B1115" t="inlineStr">
+        <is>
+          <t>operacionesinmobiliarias@proyectosyurbanizaciones.com olgapatriciaruizpineda77@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1115" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1115" t="inlineStr">
+        <is>
+          <t>26102023789886</t>
+        </is>
+      </c>
+      <c r="E1115" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1115" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1115" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1115" t="inlineStr"/>
+      <c r="I1115" t="inlineStr">
+        <is>
+          <t>754</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" t="inlineStr">
+        <is>
+          <t>818</t>
+        </is>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>julianc.avilsamoreno@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1116" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1116" t="inlineStr">
+        <is>
+          <t>26102023789916</t>
+        </is>
+      </c>
+      <c r="E1116" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1116" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1116" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1116" t="inlineStr"/>
+      <c r="I1116" t="inlineStr">
+        <is>
+          <t>818</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" t="inlineStr">
+        <is>
+          <t>877</t>
+        </is>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>gerencia@exiagricola.com</t>
+        </is>
+      </c>
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1117" t="inlineStr">
+        <is>
+          <t>26102023789932</t>
+        </is>
+      </c>
+      <c r="E1117" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1117" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1117" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1117" t="inlineStr"/>
+      <c r="I1117" t="inlineStr">
+        <is>
+          <t>877</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" t="inlineStr">
+        <is>
+          <t>900</t>
+        </is>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>alandeza@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1118" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1118" t="inlineStr">
+        <is>
+          <t>26102023789955</t>
+        </is>
+      </c>
+      <c r="E1118" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1118" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1118" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1118" t="inlineStr"/>
+      <c r="I1118" t="inlineStr">
+        <is>
+          <t>900</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" t="inlineStr">
+        <is>
+          <t>643</t>
+        </is>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>umv@marval.com.co camilo.vargas.silva@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1119" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1119" t="inlineStr">
+        <is>
+          <t>26102023789984</t>
+        </is>
+      </c>
+      <c r="E1119" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1119" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1119" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1119" t="inlineStr"/>
+      <c r="I1119" t="inlineStr">
+        <is>
+          <t>643</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" t="inlineStr">
+        <is>
+          <t>946</t>
+        </is>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>henry_latino20@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1120" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1120" t="inlineStr">
+        <is>
+          <t>26102023790013</t>
+        </is>
+      </c>
+      <c r="E1120" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1120" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1120" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1120" t="inlineStr"/>
+      <c r="I1120" t="inlineStr">
+        <is>
+          <t>946</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" t="inlineStr">
+        <is>
+          <t>837</t>
+        </is>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>taller.jaimeramirez@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1121" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1121" t="inlineStr">
+        <is>
+          <t>26102023790032</t>
+        </is>
+      </c>
+      <c r="E1121" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1121" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1121" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1121" t="inlineStr"/>
+      <c r="I1121" t="inlineStr">
+        <is>
+          <t>837</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" t="inlineStr">
+        <is>
+          <t>906</t>
+        </is>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>gustitortascoffe@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1122" t="inlineStr">
+        <is>
+          <t>26102023790050</t>
+        </is>
+      </c>
+      <c r="E1122" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1122" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1122" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1122" t="inlineStr"/>
+      <c r="I1122" t="inlineStr">
+        <is>
+          <t>906</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" t="inlineStr">
+        <is>
+          <t>198</t>
+        </is>
+      </c>
+      <c r="B1123" t="inlineStr">
+        <is>
+          <t>MARIACRISTINADERAMIREZ@GMAIL.COM</t>
+        </is>
+      </c>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1123" t="inlineStr">
+        <is>
+          <t>26102023790557</t>
+        </is>
+      </c>
+      <c r="E1123" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1123" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1123" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1123" t="inlineStr"/>
+      <c r="I1123" t="inlineStr">
+        <is>
+          <t>198</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>791</t>
+        </is>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>lilibo1963@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1124" t="inlineStr">
+        <is>
+          <t>26102023790591</t>
+        </is>
+      </c>
+      <c r="E1124" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1124" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1124" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1124" t="inlineStr"/>
+      <c r="I1124" t="inlineStr">
+        <is>
+          <t>791</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>857</t>
+        </is>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>ligiadcarmen71@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1125" t="inlineStr">
+        <is>
+          <t>26102023790620</t>
+        </is>
+      </c>
+      <c r="E1125" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1125" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1125" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1125" t="inlineStr"/>
+      <c r="I1125" t="inlineStr">
+        <is>
+          <t>857</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>894</t>
+        </is>
+      </c>
+      <c r="B1126" t="inlineStr">
+        <is>
+          <t>castanedao@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1126" t="inlineStr">
+        <is>
+          <t>26102023790643</t>
+        </is>
+      </c>
+      <c r="E1126" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1126" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1126" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1126" t="inlineStr"/>
+      <c r="I1126" t="inlineStr">
+        <is>
+          <t>894</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>878</t>
+        </is>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>esteban02006@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1127" t="inlineStr">
+        <is>
+          <t>26102023790669</t>
+        </is>
+      </c>
+      <c r="E1127" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1127" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1127" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1127" t="inlineStr"/>
+      <c r="I1127" t="inlineStr">
+        <is>
+          <t>878</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>879</t>
+        </is>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>raulgonzalez0176@yahoo.com</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1128" t="inlineStr">
+        <is>
+          <t>26102023790684</t>
+        </is>
+      </c>
+      <c r="E1128" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1128" t="inlineStr"/>
+      <c r="I1128" t="inlineStr">
+        <is>
+          <t>879</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>896</t>
+        </is>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>alvitobv@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1129" t="inlineStr">
+        <is>
+          <t>26102023790708</t>
+        </is>
+      </c>
+      <c r="E1129" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1129" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1129" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1129" t="inlineStr"/>
+      <c r="I1129" t="inlineStr">
+        <is>
+          <t>896</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>958</t>
+        </is>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>miguel-0108@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1130" t="inlineStr">
+        <is>
+          <t>26102023790728</t>
+        </is>
+      </c>
+      <c r="E1130" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1130" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1130" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1130" t="inlineStr"/>
+      <c r="I1130" t="inlineStr">
+        <is>
+          <t>958</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>637</t>
+        </is>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tati1102cruz@hotmail.com </t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1131" t="inlineStr">
+        <is>
+          <t>26102023791243</t>
+        </is>
+      </c>
+      <c r="E1131" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1131" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1131" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1131" t="inlineStr"/>
+      <c r="I1131" t="inlineStr">
+        <is>
+          <t>637</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="inlineStr">
+        <is>
+          <t>650</t>
+        </is>
+      </c>
+      <c r="B1132" t="inlineStr">
+        <is>
+          <t>lsrs.laura@hotmail.com umv@marval.com.co</t>
+        </is>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1132" t="inlineStr">
+        <is>
+          <t>26102023791275</t>
+        </is>
+      </c>
+      <c r="E1132" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1132" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1132" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1132" t="inlineStr"/>
+      <c r="I1132" t="inlineStr">
+        <is>
+          <t>650</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="inlineStr">
+        <is>
+          <t>651</t>
+        </is>
+      </c>
+      <c r="B1133" t="inlineStr">
+        <is>
+          <t>lauranrp@gmail.com umv@marval.com.co</t>
+        </is>
+      </c>
+      <c r="C1133" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1133" t="inlineStr">
+        <is>
+          <t>26102023791343</t>
+        </is>
+      </c>
+      <c r="E1133" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1133" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1133" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1133" t="inlineStr"/>
+      <c r="I1133" t="inlineStr">
+        <is>
+          <t>651</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>773</t>
+        </is>
+      </c>
+      <c r="B1134" t="inlineStr">
+        <is>
+          <t>edwardocogua@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1134" t="inlineStr">
+        <is>
+          <t>26102023796805</t>
+        </is>
+      </c>
+      <c r="E1134" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1134" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1134" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1134" t="inlineStr"/>
+      <c r="I1134" t="inlineStr">
+        <is>
+          <t>773</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" t="inlineStr">
+        <is>
+          <t>149</t>
+        </is>
+      </c>
+      <c r="B1135" t="inlineStr">
+        <is>
+          <t>jmattsanchez@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1135" t="inlineStr">
+        <is>
+          <t>26102023796850</t>
+        </is>
+      </c>
+      <c r="E1135" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1135" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1135" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1135" t="inlineStr"/>
+      <c r="I1135" t="inlineStr">
+        <is>
+          <t>149</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" t="inlineStr">
+        <is>
+          <t>167</t>
+        </is>
+      </c>
+      <c r="B1136" t="inlineStr">
+        <is>
+          <t>angelagutip7910@outlook.com</t>
+        </is>
+      </c>
+      <c r="C1136" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1136" t="inlineStr">
+        <is>
+          <t>26102023796881</t>
+        </is>
+      </c>
+      <c r="E1136" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1136" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1136" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1136" t="inlineStr"/>
+      <c r="I1136" t="inlineStr">
+        <is>
+          <t>167</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" t="inlineStr">
+        <is>
+          <t>792</t>
+        </is>
+      </c>
+      <c r="B1137" t="inlineStr">
+        <is>
+          <t>javi39upn@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1137" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1137" t="inlineStr">
+        <is>
+          <t>26102023796908</t>
+        </is>
+      </c>
+      <c r="E1137" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1137" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1137" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1137" t="inlineStr"/>
+      <c r="I1137" t="inlineStr">
+        <is>
+          <t>792</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" t="inlineStr">
+        <is>
+          <t>871</t>
+        </is>
+      </c>
+      <c r="B1138" t="inlineStr">
+        <is>
+          <t>mariaeugeniadallos@yahoo.es</t>
+        </is>
+      </c>
+      <c r="C1138" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1138" t="inlineStr">
+        <is>
+          <t>26102023796961</t>
+        </is>
+      </c>
+      <c r="E1138" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1138" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1138" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1138" t="inlineStr"/>
+      <c r="I1138" t="inlineStr">
+        <is>
+          <t>871</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="inlineStr">
+        <is>
+          <t>873</t>
+        </is>
+      </c>
+      <c r="B1139" t="inlineStr">
+        <is>
+          <t>philip-74@hotmail.com angie1023k@gmai.com dianar0102@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1139" t="inlineStr">
+        <is>
+          <t>26102023797165</t>
+        </is>
+      </c>
+      <c r="E1139" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1139" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1139" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1139" t="inlineStr"/>
+      <c r="I1139" t="inlineStr">
+        <is>
+          <t>873</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="inlineStr">
+        <is>
+          <t>892</t>
+        </is>
+      </c>
+      <c r="B1140" t="inlineStr">
+        <is>
+          <t>gomezjaimealberto@gmail.com leogomez239@hotmail.com pagovallejo@hotmail.com olgomez11@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="D1140" t="inlineStr">
+        <is>
+          <t>26102023797208</t>
+        </is>
+      </c>
+      <c r="E1140" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1140" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1140" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1140" t="inlineStr"/>
+      <c r="I1140" t="inlineStr">
+        <is>
+          <t>892</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="inlineStr">
+        <is>
+          <t>903</t>
+        </is>
+      </c>
+      <c r="B1141" t="inlineStr">
+        <is>
+          <t>corinaduque@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1141" t="inlineStr">
+        <is>
+          <t>26102023797823</t>
+        </is>
+      </c>
+      <c r="E1141" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1141" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1141" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1141" t="inlineStr"/>
+      <c r="I1141" t="inlineStr">
+        <is>
+          <t>903</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="inlineStr">
+        <is>
+          <t>916</t>
+        </is>
+      </c>
+      <c r="B1142" t="inlineStr">
+        <is>
+          <t>josepenabogados@gmail.com eulisespena326@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>Tolima</t>
+        </is>
+      </c>
+      <c r="D1142" t="inlineStr">
+        <is>
+          <t>26102023798007</t>
+        </is>
+      </c>
+      <c r="E1142" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1142" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1142" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1142" t="inlineStr"/>
+      <c r="I1142" t="inlineStr">
+        <is>
+          <t>916</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="inlineStr">
+        <is>
+          <t>924</t>
+        </is>
+      </c>
+      <c r="B1143" t="inlineStr">
+        <is>
+          <t>fiurescarfc@gmail.com nieves-gurrero12@hotmail.com fivrescarfc@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1143" t="inlineStr">
+        <is>
+          <t>26102023798041</t>
+        </is>
+      </c>
+      <c r="E1143" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1143" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1143" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1143" t="inlineStr"/>
+      <c r="I1143" t="inlineStr">
+        <is>
+          <t>924</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="inlineStr">
+        <is>
+          <t>934</t>
+        </is>
+      </c>
+      <c r="B1144" t="inlineStr">
+        <is>
+          <t>delgado.alirio@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1144" t="inlineStr">
+        <is>
+          <t>26102023798451</t>
+        </is>
+      </c>
+      <c r="E1144" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1144" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1144" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1144" t="inlineStr"/>
+      <c r="I1144" t="inlineStr">
+        <is>
+          <t>934</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="inlineStr">
+        <is>
+          <t>937</t>
+        </is>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>gutierrezstrella99@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1145" t="inlineStr">
+        <is>
+          <t>26102023798472</t>
+        </is>
+      </c>
+      <c r="E1145" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1145" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1145" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1145" t="inlineStr"/>
+      <c r="I1145" t="inlineStr">
+        <is>
+          <t>937</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>957</t>
+        </is>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>contabilidad@redetronix.com</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1146" t="inlineStr">
+        <is>
+          <t>26102023798510</t>
+        </is>
+      </c>
+      <c r="E1146" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1146" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1146" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1146" t="inlineStr"/>
+      <c r="I1146" t="inlineStr">
+        <is>
+          <t>957</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>766</t>
+        </is>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>marcelitalann@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1147" t="inlineStr">
+        <is>
+          <t>26102023798739</t>
+        </is>
+      </c>
+      <c r="E1147" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1147" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1147" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1147" t="inlineStr"/>
+      <c r="I1147" t="inlineStr">
+        <is>
+          <t>766</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>876</t>
+        </is>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>toromarcelo@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1148" t="inlineStr">
+        <is>
+          <t>26102023798942</t>
+        </is>
+      </c>
+      <c r="E1148" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1148" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1148" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1148" t="inlineStr"/>
+      <c r="I1148" t="inlineStr">
+        <is>
+          <t>876</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>918</t>
+        </is>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>yo-lis69@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1149" t="inlineStr">
+        <is>
+          <t>26102023799012</t>
+        </is>
+      </c>
+      <c r="E1149" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1149" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1149" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1149" t="inlineStr"/>
+      <c r="I1149" t="inlineStr">
+        <is>
+          <t>918</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>936</t>
+        </is>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>maderclav@hotmail.com contactonvogim@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1150" t="inlineStr">
+        <is>
+          <t>26102023799050</t>
+        </is>
+      </c>
+      <c r="E1150" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1150" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1150" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1150" t="inlineStr"/>
+      <c r="I1150" t="inlineStr">
+        <is>
+          <t>936</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>960</t>
+        </is>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>gpd_63@yahoo.es</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1151" t="inlineStr">
+        <is>
+          <t>26102023799079</t>
+        </is>
+      </c>
+      <c r="E1151" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1151" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1151" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1151" t="inlineStr"/>
+      <c r="I1151" t="inlineStr">
+        <is>
+          <t>960</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>778</t>
+        </is>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>nandopsarmiento@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1152" t="inlineStr">
+        <is>
+          <t>26102023799666</t>
+        </is>
+      </c>
+      <c r="E1152" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1152" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1152" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1152" t="inlineStr"/>
+      <c r="I1152" t="inlineStr">
+        <is>
+          <t>778</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>847</t>
+        </is>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>wocpcruz@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1153" t="inlineStr">
+        <is>
+          <t>26102023798665</t>
+        </is>
+      </c>
+      <c r="E1153" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1153" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1153" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1153" t="inlineStr"/>
+      <c r="I1153" t="inlineStr">
+        <is>
+          <t>847</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>406</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>majimenez_867@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1154" t="inlineStr">
+        <is>
+          <t>26102023799159</t>
+        </is>
+      </c>
+      <c r="E1154" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1154" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1154" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1154" t="inlineStr"/>
+      <c r="I1154" t="inlineStr">
+        <is>
+          <t>406</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>908</t>
+        </is>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>guillerveca@hotmail.com guillervega@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1155" t="inlineStr">
+        <is>
+          <t>26102023799264</t>
+        </is>
+      </c>
+      <c r="E1155" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1155" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1155" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1155" t="inlineStr"/>
+      <c r="I1155" t="inlineStr">
+        <is>
+          <t>908</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>683</t>
+        </is>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>epinzont@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1156" t="inlineStr">
+        <is>
+          <t>26102023799463</t>
+        </is>
+      </c>
+      <c r="E1156" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1156" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1156" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1156" t="inlineStr"/>
+      <c r="I1156" t="inlineStr">
+        <is>
+          <t>683</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>935</t>
+        </is>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>brayanmonroy95@hotmail.com analucindacortes@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1157" t="inlineStr">
+        <is>
+          <t>26102023799510</t>
+        </is>
+      </c>
+      <c r="E1157" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1157" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1157" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1157" t="inlineStr"/>
+      <c r="I1157" t="inlineStr">
+        <is>
+          <t>935</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>858</t>
+        </is>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>carmengaona1708@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1158" t="inlineStr">
+        <is>
+          <t>26102023799545</t>
+        </is>
+      </c>
+      <c r="E1158" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1158" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1158" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1158" t="inlineStr"/>
+      <c r="I1158" t="inlineStr">
+        <is>
+          <t>858</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="inlineStr">
+        <is>
+          <t>156</t>
+        </is>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>gavilagraficos@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1159" t="inlineStr">
+        <is>
+          <t>26102023799615</t>
+        </is>
+      </c>
+      <c r="E1159" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1159" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1159" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1159" t="inlineStr"/>
+      <c r="I1159" t="inlineStr">
+        <is>
+          <t>156</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="inlineStr">
+        <is>
+          <t>451</t>
+        </is>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>ubaldovega892@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1160" t="inlineStr">
+        <is>
+          <t>26102023801351</t>
+        </is>
+      </c>
+      <c r="E1160" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1160" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1160" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1160" t="inlineStr"/>
+      <c r="I1160" t="inlineStr">
+        <is>
+          <t>451</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="inlineStr">
+        <is>
+          <t>710</t>
+        </is>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>gerencia.juridica@cobracs.com.co</t>
+        </is>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1161" t="inlineStr">
+        <is>
+          <t>26102023801399</t>
+        </is>
+      </c>
+      <c r="E1161" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1161" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1161" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1161" t="inlineStr"/>
+      <c r="I1161" t="inlineStr">
+        <is>
+          <t>710</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>787</t>
+        </is>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>joserafael2110@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1162" t="inlineStr">
+        <is>
+          <t>26102023801447</t>
+        </is>
+      </c>
+      <c r="E1162" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1162" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1162" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1162" t="inlineStr"/>
+      <c r="I1162" t="inlineStr">
+        <is>
+          <t>787</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="inlineStr">
+        <is>
+          <t>794</t>
+        </is>
+      </c>
+      <c r="B1163" t="inlineStr">
+        <is>
+          <t>aida.castro1583@gmail.com operacionesinmobiliarias@proyectosyurbanizaciones.com</t>
+        </is>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1163" t="inlineStr">
+        <is>
+          <t>26102023801499</t>
+        </is>
+      </c>
+      <c r="E1163" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1163" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1163" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1163" t="inlineStr"/>
+      <c r="I1163" t="inlineStr">
+        <is>
+          <t>794</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="inlineStr">
+        <is>
+          <t>893</t>
+        </is>
+      </c>
+      <c r="B1164" t="inlineStr">
+        <is>
+          <t>yoliconi.26@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1164" t="inlineStr">
+        <is>
+          <t>26102023801769</t>
+        </is>
+      </c>
+      <c r="E1164" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1164" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1164" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1164" t="inlineStr"/>
+      <c r="I1164" t="inlineStr">
+        <is>
+          <t>893</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" t="inlineStr">
+        <is>
+          <t>942</t>
+        </is>
+      </c>
+      <c r="B1165" t="inlineStr">
+        <is>
+          <t>comercializadorajapaca@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C1165" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1165" t="inlineStr">
+        <is>
+          <t>26102023801812</t>
+        </is>
+      </c>
+      <c r="E1165" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1165" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1165" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1165" t="inlineStr"/>
+      <c r="I1165" t="inlineStr">
+        <is>
+          <t>942</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" t="inlineStr">
+        <is>
+          <t>790</t>
+        </is>
+      </c>
+      <c r="B1166" t="inlineStr">
+        <is>
+          <t>caprietoabogado@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1166" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1166" t="inlineStr">
+        <is>
+          <t>26102023802958</t>
+        </is>
+      </c>
+      <c r="E1166" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1166" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1166" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1166" t="inlineStr"/>
+      <c r="I1166" t="inlineStr">
+        <is>
+          <t>790</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" t="inlineStr">
+        <is>
+          <t>967</t>
+        </is>
+      </c>
+      <c r="B1167" t="inlineStr">
+        <is>
+          <t>marysierrasantana@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1167" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1167" t="inlineStr">
+        <is>
+          <t>26102023803015</t>
+        </is>
+      </c>
+      <c r="E1167" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F1167" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G1167" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H1167" t="inlineStr"/>
+      <c r="I1167" t="inlineStr">
+        <is>
+          <t>967</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" t="inlineStr">
+        <is>
+          <t>920</t>
+        </is>
+      </c>
+      <c r="B1168" t="inlineStr">
+        <is>
+          <t>cesara.torres123@gmail.com ceidyjuana@gmail.com</t>
+        </is>
+      </c>
+      <c r="C1168" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="D1168" t="inlineStr">
+        <is>
+          <t>26102023805429</t>
+        </is>
+      </c>
+      <c r="E1168" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="F1168" t="inlineStr"/>
+      <c r="G1168" t="inlineStr"/>
+      <c r="H1168" t="inlineStr"/>
+      <c r="I1168" t="inlineStr">
+        <is>
+          <t>920</t>
         </is>
       </c>
     </row>

</xml_diff>